<commit_message>
It may be good
</commit_message>
<xml_diff>
--- a/excel/matrix_cohen.xlsx
+++ b/excel/matrix_cohen.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="mistral_Rag" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -878,9 +879,477 @@
       <c r="J11" t="n">
         <v>1</v>
       </c>
+      <c r="L11" t="n">
+        <v>0.02948847993044487</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.008474729732176811</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.008474729732176811</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Breakpoint1: the rag is correctly running and the output matrix and perf are correctly managed
</commit_message>
<xml_diff>
--- a/excel/matrix_cohen.xlsx
+++ b/excel/matrix_cohen.xlsx
@@ -8,7 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="mistral_Rag" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="phi4_Rag" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="llama3.3_Rag" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="mistral_No_rag" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="mistral_Rag" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="llama3.3_No_rag" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Rag_keyword_Rag" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mistral_Rag_keyword" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="phi4_Rag_keyword" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="phi4_No_rag" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="llama3.3_Rag_keyword" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,6 +435,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -493,22 +515,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -517,13 +539,13 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="3">
@@ -536,10 +558,10 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -560,10 +582,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="L3" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="4">
@@ -576,10 +598,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -600,10 +622,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L4" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="5">
@@ -616,13 +638,13 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -640,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="6">
@@ -656,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -665,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -674,16 +696,16 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="7">
@@ -696,7 +718,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -708,22 +730,22 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="L7" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="8">
@@ -736,10 +758,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -748,22 +770,22 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="L8" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="9">
@@ -776,34 +798,34 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="L9" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="10">
@@ -828,22 +850,22 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="L10" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
       </c>
     </row>
     <row r="11">
@@ -853,34 +875,503 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02948847993044487</v>
+        <v>0.3782947847569398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>13</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>21</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.7519998311488212</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>33</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D11" t="n">
+        <v>51</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" t="n">
+        <v>47</v>
+      </c>
+      <c r="I11" t="n">
+        <v>24</v>
+      </c>
+      <c r="J11" t="n">
+        <v>31</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0.7519998311488212</v>
       </c>
     </row>
   </sheetData>
@@ -961,13 +1452,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -976,22 +1467,22 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="L2" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="3">
@@ -1004,7 +1495,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1028,10 +1519,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="L3" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="4">
@@ -1041,13 +1532,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1068,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L4" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="5">
@@ -1090,7 +1581,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1108,10 +1599,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="6">
@@ -1121,10 +1612,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1133,10 +1624,10 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1148,10 +1639,10 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L6" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="7">
@@ -1161,7 +1652,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -1176,7 +1667,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -1188,10 +1679,10 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="8">
@@ -1207,31 +1698,31 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L8" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="9">
@@ -1241,37 +1732,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="L9" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="10">
@@ -1281,7 +1772,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1299,19 +1790,19 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="L10" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
       </c>
     </row>
     <row r="11">
@@ -1321,35 +1812,3310 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="inlineStr"/>
+        <v>32</v>
+      </c>
       <c r="L11" t="n">
-        <v>0.008474729732176811</v>
+        <v>0.5636505211037015</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>32</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>11</v>
+      </c>
+      <c r="I9" t="n">
+        <v>17</v>
+      </c>
+      <c r="J9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>19</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>37</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D11" t="n">
+        <v>51</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" t="n">
+        <v>19</v>
+      </c>
+      <c r="J11" t="n">
+        <v>29</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7128168390889362</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>21</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>31</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>13</v>
+      </c>
+      <c r="C9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>43</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>22</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>43</v>
+      </c>
+      <c r="C11" t="n">
+        <v>65</v>
+      </c>
+      <c r="D11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>19</v>
+      </c>
+      <c r="H11" t="n">
+        <v>16</v>
+      </c>
+      <c r="I11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.3154675211185552</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>29</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>32</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" t="n">
+        <v>29</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>21</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>38</v>
+      </c>
+      <c r="C11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" t="n">
+        <v>49</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" t="n">
+        <v>42</v>
+      </c>
+      <c r="I11" t="n">
+        <v>41</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.6367390153520383</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" t="n">
+        <v>42</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>29</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>12</v>
+      </c>
+      <c r="I9" t="n">
+        <v>14</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>14</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" t="n">
+        <v>33</v>
+      </c>
+      <c r="D11" t="n">
+        <v>54</v>
+      </c>
+      <c r="E11" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>17</v>
+      </c>
+      <c r="H11" t="n">
+        <v>47</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" t="n">
+        <v>21</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.5948361052122538</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>24</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>42</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>29</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>12</v>
+      </c>
+      <c r="I9" t="n">
+        <v>13</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>12</v>
+      </c>
+      <c r="K10" t="n">
+        <v>22</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="n">
+        <v>31</v>
+      </c>
+      <c r="D11" t="n">
+        <v>54</v>
+      </c>
+      <c r="E11" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" t="n">
+        <v>47</v>
+      </c>
+      <c r="I11" t="n">
+        <v>19</v>
+      </c>
+      <c r="J11" t="n">
+        <v>17</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.5805421977698914</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>22</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>11</v>
+      </c>
+      <c r="I9" t="n">
+        <v>29</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" t="n">
+        <v>22</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31</v>
+      </c>
+      <c r="C11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D11" t="n">
+        <v>57</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>17</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" t="n">
+        <v>37</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.6844292870084195</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>34</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>23</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>31</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K9" t="n">
+        <v>41</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>21</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6393230744375783</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>26</v>
+      </c>
+      <c r="C11" t="n">
+        <v>31</v>
+      </c>
+      <c r="D11" t="n">
+        <v>31</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23</v>
+      </c>
+      <c r="H11" t="n">
+        <v>34</v>
+      </c>
+      <c r="I11" t="n">
+        <v>21</v>
+      </c>
+      <c r="J11" t="n">
+        <v>35</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.6393230744375783</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
debate hybrid, mistral comme orchestrateur
</commit_message>
<xml_diff>
--- a/excel/matrix_cohen.xlsx
+++ b/excel/matrix_cohen.xlsx
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="3">
@@ -549,7 +549,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -573,10 +573,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="4">
@@ -592,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -613,10 +613,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="5">
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="6">
@@ -696,7 +696,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="7">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -721,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -733,10 +733,10 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="8">
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -773,10 +773,10 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="9">
@@ -795,7 +795,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -804,19 +804,19 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L9" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="10">
@@ -856,7 +856,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
     <row r="11">
@@ -866,35 +866,35 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.00423728813559322</v>
+        <v>0.05812477330431627</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Breakpoint : Here I defended. The actual code is about the hybrid architecture with the same instance of the same LLM(easily)
</commit_message>
<xml_diff>
--- a/excel/matrix_cohen.xlsx
+++ b/excel/matrix_cohen.xlsx
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="3">
@@ -549,7 +549,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -573,10 +573,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="4">
@@ -592,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -613,10 +613,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="5">
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="6">
@@ -696,7 +696,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="7">
@@ -721,22 +721,22 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
         <v>1</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>2</v>
-      </c>
       <c r="L7" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="8">
@@ -749,10 +749,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -773,10 +773,10 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="9">
@@ -786,37 +786,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" t="n">
-        <v>3</v>
-      </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="L9" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="10">
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -853,10 +853,10 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
     <row r="11">
@@ -866,13 +866,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -881,20 +881,20 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" t="n">
         <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>9</v>
-      </c>
-      <c r="I11" t="n">
-        <v>3</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.05812477330431627</v>
+        <v>0.06507166603084637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Work on the output format modification
</commit_message>
<xml_diff>
--- a/excel/matrix_cohen.xlsx
+++ b/excel/matrix_cohen.xlsx
@@ -13,6 +13,8 @@
     <sheet name="llama3.3_Rag_keyword" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="llama3.3_Rag" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Rag_phi4_rag" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Rag_mistral_rag" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Rag_llama3_3_rag" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1932,14 +1934,952 @@
           <t>MonCal.Interpret</t>
         </is>
       </c>
+      <c r="B2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr"/>
+      <c r="L11" s="0" t="n">
+        <v>0.01271232479808772</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr"/>
+      <c r="L11" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1957,13 +2897,13 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
         <v>23</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="3">
@@ -2003,7 +2943,7 @@
         <v>26</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="4">
@@ -2016,10 +2956,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -2043,7 +2983,7 @@
         <v>51</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="5">
@@ -2083,7 +3023,7 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="6">
@@ -2093,7 +3033,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -2105,7 +3045,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -2123,7 +3063,7 @@
         <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="7">
@@ -2133,7 +3073,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -2148,7 +3088,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -2157,13 +3097,13 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="8">
@@ -2179,7 +3119,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -2188,22 +3128,22 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>34</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="9">
@@ -2213,37 +3153,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I9" t="n">
         <v>25</v>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
         <v>46</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="10">
@@ -2271,19 +3211,19 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K10" t="n">
         <v>23</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
     <row r="11">
@@ -2293,35 +3233,35 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C11" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" t="n">
         <v>57</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H11" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I11" t="n">
+        <v>27</v>
+      </c>
+      <c r="J11" t="n">
         <v>29</v>
-      </c>
-      <c r="J11" t="n">
-        <v>36</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.7760862200389599</v>
+        <v>0.8059002922614258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>